<commit_message>
test coverage using JIRA
</commit_message>
<xml_diff>
--- a/Test_Cases (1).xlsx
+++ b/Test_Cases (1).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="6200" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Login Module" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="265">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -529,7 +529,7 @@
     <t>TC_PIM_010</t>
   </si>
   <si>
-    <t>Verify First Name field rejects numeric/special characters</t>
+    <t>Verify First Name field rejects numeric/special characters (NEGATIVE TESTING)</t>
   </si>
   <si>
     <t>On PIM &gt; Add Employee</t>
@@ -590,6 +590,75 @@
   </si>
   <si>
     <t>Form resets/does not retain unsaved data</t>
+  </si>
+  <si>
+    <t>TC_PIM_013</t>
+  </si>
+  <si>
+    <t>Verify updating job details, Employment Status, Sub Unit, Supervisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIM → open an existing employee 
+</t>
+  </si>
+  <si>
+    <t>1. open an existing employee
+2. edit field job, employment status etc
+3. Save</t>
+  </si>
+  <si>
+    <t>All the changes would be displayed in the employee record</t>
+  </si>
+  <si>
+    <t>changes saved successfully and showing in employee record</t>
+  </si>
+  <si>
+    <t>TC_PIM_014</t>
+  </si>
+  <si>
+    <t>Verify deleting multiple employee record</t>
+  </si>
+  <si>
+    <t>1. open an existing employee
+2. select multiple employee to delete
+3. click delete</t>
+  </si>
+  <si>
+    <t>All the selected employees should be deleted</t>
+  </si>
+  <si>
+    <t>employees deleted</t>
+  </si>
+  <si>
+    <t>TC_PIM_015</t>
+  </si>
+  <si>
+    <t>Cancel delete confirmation (record should remain)</t>
+  </si>
+  <si>
+    <t>1. open an existing employee
+2. select multiple employee to delete
+3. click delete, then cancel delete confirmation</t>
+  </si>
+  <si>
+    <t>All the selected employees should be remained</t>
+  </si>
+  <si>
+    <t>employees were remained in the list</t>
+  </si>
+  <si>
+    <t>TC_PIM_016</t>
+  </si>
+  <si>
+    <t>Verify searching for an employee by id</t>
+  </si>
+  <si>
+    <t>1. Navigate to PIM &gt; Employee List
+2. Enter employee id in search field
+3. Click Search</t>
+  </si>
+  <si>
+    <t>Employee id: (existing employee's id)</t>
   </si>
   <si>
     <t>TC_LEAVE_001</t>
@@ -1522,7 +1591,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1535,6 +1604,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2279,10 +2351,10 @@
       <c r="G12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="7" t="s">
         <v>18</v>
       </c>
       <c r="J12" s="3" t="s">
@@ -2311,7 +2383,7 @@
       <c r="G13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="6" t="s">
         <v>85</v>
       </c>
       <c r="I13" s="3" t="s">
@@ -2330,7 +2402,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -2472,7 +2544,7 @@
       <c r="G4" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="8" t="s">
         <v>108</v>
       </c>
       <c r="I4" s="3" t="s">
@@ -2574,10 +2646,10 @@
       <c r="F7" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="8" t="s">
         <v>127</v>
       </c>
       <c r="I7" s="3" t="s">
@@ -2797,6 +2869,137 @@
         <v>56</v>
       </c>
       <c r="K13" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" customFormat="1" ht="58" spans="1:11">
+      <c r="A14" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" ht="58" spans="1:11">
+      <c r="A15" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" customFormat="1" ht="58" spans="1:11">
+      <c r="A16" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" customFormat="1" ht="60" customHeight="1" spans="1:11">
+      <c r="A17" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" s="3" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2861,28 +3064,28 @@
     </row>
     <row r="2" ht="60" customHeight="1" spans="1:11">
       <c r="A2" s="3" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>18</v>
@@ -2893,28 +3096,28 @@
     </row>
     <row r="3" ht="60" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>18</v>
@@ -2925,28 +3128,28 @@
     </row>
     <row r="4" ht="60" customHeight="1" spans="1:11">
       <c r="A4" s="3" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>18</v>
@@ -2957,28 +3160,28 @@
     </row>
     <row r="5" ht="60" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>86</v>
@@ -2989,28 +3192,28 @@
     </row>
     <row r="6" ht="60" customHeight="1" spans="1:11">
       <c r="A6" s="3" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>196</v>
+        <v>216</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>18</v>
@@ -3021,28 +3224,28 @@
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:11">
       <c r="A7" s="3" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>72</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>204</v>
+        <v>224</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>205</v>
+        <v>225</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>18</v>
@@ -3053,28 +3256,28 @@
     </row>
     <row r="8" ht="60" customHeight="1" spans="1:11">
       <c r="A8" s="3" t="s">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>207</v>
+        <v>227</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>209</v>
+        <v>229</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>72</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>86</v>
@@ -3085,28 +3288,28 @@
     </row>
     <row r="9" ht="60" customHeight="1" spans="1:11">
       <c r="A9" s="3" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>72</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>216</v>
+        <v>236</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>86</v>
@@ -3117,28 +3320,28 @@
     </row>
     <row r="10" ht="60" customHeight="1" spans="1:11">
       <c r="A10" s="3" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>72</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>18</v>
@@ -3149,28 +3352,28 @@
     </row>
     <row r="11" ht="60" customHeight="1" spans="1:11">
       <c r="A11" s="3" t="s">
-        <v>223</v>
+        <v>243</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>226</v>
+        <v>246</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>228</v>
+        <v>248</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>229</v>
+        <v>249</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>18</v>
@@ -3181,28 +3384,28 @@
     </row>
     <row r="12" ht="60" customHeight="1" spans="1:11">
       <c r="A12" s="3" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>232</v>
+        <v>252</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>234</v>
+        <v>254</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>18</v>
@@ -3213,28 +3416,28 @@
     </row>
     <row r="13" ht="133" customHeight="1" spans="1:11">
       <c r="A13" s="3" t="s">
-        <v>237</v>
+        <v>257</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>242</v>
+        <v>262</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>18</v>
@@ -3243,7 +3446,7 @@
         <v>37</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>